<commit_message>
fix: make funding site refresh latest data
</commit_message>
<xml_diff>
--- a/site/近期融资公司追踪.xlsx
+++ b/site/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R54fc4dda98324605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R42f27c937d0b4fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Rd3e570be538e4915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R0c8ccae558f5444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rabd730b84bea4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Rba3a3a15413a4830"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2694,7 +2694,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46272.41982944444</x:v>
+        <x:v>46272.42526790509</x:v>
       </x:c>
       <x:c r="B2" t="n">
         <x:v>43</x:v>

</xml_diff>